<commit_message>
Weekly Pulse: cream This Week tiles, noise bucket fixes, tp-num white
</commit_message>
<xml_diff>
--- a/Final Data Files/Team Pulse/EDEN_CO_Weekly_Status.xlsx
+++ b/Final Data Files/Team Pulse/EDEN_CO_Weekly_Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bf0016d8e2d976c3/eden-co-brain/data/ceo dashboard/build/Final Data Files/Team Pulse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="498" documentId="11_5BE35CD9EAE0455C5359B5B6448765289977FBF5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F75E168B-41D2-4AC6-BA36-781DDAC30F63}"/>
+  <xr:revisionPtr revIDLastSave="499" documentId="11_5BE35CD9EAE0455C5359B5B6448765289977FBF5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16E12C85-D739-482F-A661-2790550C118A}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" firstSheet="3" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jon" sheetId="2" r:id="rId1"/>
@@ -5173,7 +5173,7 @@
         <v>41</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Dashboard session 30 Mar: 5 major additions
- Update status icon + data source popout in toolbar
- Team Pulse: 2-column layout matching spreadsheet order
- Platforms tab: split Sales Channels / Corporate sections
- Operations: BoM matrix + hamper view from BoM.xlsx (41 products)
- Socials: Dream Value Equation post analyser + platform priority grid
</commit_message>
<xml_diff>
--- a/Final Data Files/Team Pulse/EDEN_CO_Weekly_Status.xlsx
+++ b/Final Data Files/Team Pulse/EDEN_CO_Weekly_Status.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bf0016d8e2d976c3/eden-co-brain/data/ceo dashboard/build/Final Data Files/Team Pulse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="499" documentId="11_5BE35CD9EAE0455C5359B5B6448765289977FBF5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16E12C85-D739-482F-A661-2790550C118A}"/>
+  <xr:revisionPtr revIDLastSave="517" documentId="11_5BE35CD9EAE0455C5359B5B6448765289977FBF5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CCE7DF9-86A2-42B9-80EC-C1483354DD52}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" firstSheet="3" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Jon" sheetId="2" r:id="rId1"/>
-    <sheet name="Rosie" sheetId="3" r:id="rId2"/>
-    <sheet name="Edith" sheetId="4" r:id="rId3"/>
-    <sheet name="Phoebe" sheetId="5" r:id="rId4"/>
+    <sheet name="Phoebe" sheetId="5" r:id="rId1"/>
+    <sheet name="Edith" sheetId="4" r:id="rId2"/>
+    <sheet name="Rosie" sheetId="3" r:id="rId3"/>
+    <sheet name="Jon" sheetId="2" r:id="rId4"/>
     <sheet name="Concerns" sheetId="6" r:id="rId5"/>
     <sheet name="UGC Influencers" sheetId="9" r:id="rId6"/>
     <sheet name="IG Accounts" sheetId="8" r:id="rId7"/>
-    <sheet name="Core Goals" sheetId="1" state="hidden" r:id="rId8"/>
+    <sheet name="Core Goals" sheetId="1" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,9 +43,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3049" uniqueCount="1217">
-  <si>
-    <t>Jon · Business Lead · Weekly Actions</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3054" uniqueCount="1218">
+  <si>
+    <t>Phoebe - Operations · Weekly Actions</t>
   </si>
   <si>
     <t>Update your This week tasks by Friday 5pm. Mark done, on-track, blocked or overdue. Add a note if anything is not complete.</t>
@@ -78,130 +78,40 @@
     <t>2026-W13</t>
   </si>
   <si>
-    <t>Jon</t>
+    <t>Phoebe</t>
   </si>
   <si>
     <t>This week</t>
   </si>
   <si>
-    <t>Amazon Account Validation (VAT + Phone)</t>
+    <t>Support Whouse Despatch</t>
   </si>
   <si>
     <t>on-track</t>
   </si>
   <si>
-    <t>B2B - 2 key accounts/month</t>
-  </si>
-  <si>
-    <t>Contact Accountants &amp; Chase Amazon</t>
-  </si>
-  <si>
-    <t>Support Phoebe - Orders Despatch</t>
-  </si>
-  <si>
-    <t>Business Strategy &amp; Performance</t>
-  </si>
-  <si>
-    <t>Mon-Thu Practice</t>
-  </si>
-  <si>
-    <t>Teach Phoebe Invoicing</t>
-  </si>
-  <si>
-    <t>Monday Teaching</t>
-  </si>
-  <si>
-    <t>Payroll</t>
-  </si>
-  <si>
-    <t>Monday Update</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Launch New Dashboard </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monday Meeting Unveil </t>
-  </si>
-  <si>
-    <t>Finalise 2026 Product Range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GreenFingers Outstanding </t>
-  </si>
-  <si>
-    <t>Monitor International Orders</t>
-  </si>
-  <si>
-    <t>International - shipping + Amz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UPS checkin </t>
-  </si>
-  <si>
-    <t>2026-W14</t>
-  </si>
-  <si>
-    <t>GlobalCheckout Setup</t>
-  </si>
-  <si>
-    <t>Bread&amp;Jam Tickets</t>
-  </si>
-  <si>
-    <t>Buy these</t>
-  </si>
-  <si>
-    <t>Checking WIth Corp Campaigns: Virgin, PIPL, SmartCurrencyExchange</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email each Monday </t>
-  </si>
-  <si>
-    <t>PPC Check-in &amp; Ypdate</t>
-  </si>
-  <si>
-    <t>PPC - Blended ROAS 5x</t>
-  </si>
-  <si>
-    <t>Create Brochure (Inbox)</t>
-  </si>
-  <si>
-    <t>Rosie - Brand + UX + Team Support · Weekly Actions</t>
-  </si>
-  <si>
-    <t>Rosie</t>
-  </si>
-  <si>
-    <t>Chase RH Fibreboard - packaging quotes</t>
-  </si>
-  <si>
-    <t>Stock + product QA</t>
-  </si>
-  <si>
-    <t>Checkin Founder Content with Edith</t>
-  </si>
-  <si>
-    <t>Content brand QA every piece</t>
-  </si>
-  <si>
-    <t>Checkin UGC Content with Edith</t>
-  </si>
-  <si>
-    <t>Pack Gift Tubes</t>
-  </si>
-  <si>
-    <t>W/House Assemble Plan with Phoebe</t>
-  </si>
-  <si>
-    <t>Continue Despatch Training Phoebe</t>
-  </si>
-  <si>
-    <t>Team training needs - identify + act</t>
-  </si>
-  <si>
-    <t>Decide on new Product lines</t>
-  </si>
-  <si>
-    <t>Confirm Building Works</t>
+    <t>Order satisfaction + despatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goal: Teach Edith Despatch process in full by end of April </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn Admin Despatch </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goal: Teach Rosie Despatch process in full by end of April </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn Invoicing &amp; Purchase Order  </t>
+  </si>
+  <si>
+    <t>Admin &amp; Finance</t>
+  </si>
+  <si>
+    <t>Pack GiftTubes</t>
+  </si>
+  <si>
+    <t>Stock planning</t>
   </si>
   <si>
     <t>Edith - Marketing · Weekly Actions</t>
@@ -246,37 +156,127 @@
 Amends Made / Sign-off</t>
   </si>
   <si>
-    <t>Phoebe - Operations · Weekly Actions</t>
-  </si>
-  <si>
-    <t>Phoebe</t>
-  </si>
-  <si>
-    <t>Support Whouse Despatch</t>
-  </si>
-  <si>
-    <t>Order satisfaction + despatch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goal: Teach Edith Despatch process in full by end of April </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Learn Admin Despatch </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goal: Teach Rosie Despatch process in full by end of April </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Learn Invoicing &amp; Purchase Order  </t>
-  </si>
-  <si>
-    <t>Admin &amp; Finance</t>
-  </si>
-  <si>
-    <t>Pack GiftTubes</t>
-  </si>
-  <si>
-    <t>Stock planning</t>
+    <t>Rosie - Brand + UX + Team Support · Weekly Actions</t>
+  </si>
+  <si>
+    <t>Rosie</t>
+  </si>
+  <si>
+    <t>Chase RH Fibreboard - packaging quotes</t>
+  </si>
+  <si>
+    <t>Stock + product QA</t>
+  </si>
+  <si>
+    <t>Checkin Founder Content with Edith</t>
+  </si>
+  <si>
+    <t>Content brand QA every piece</t>
+  </si>
+  <si>
+    <t>Checkin UGC Content with Edith</t>
+  </si>
+  <si>
+    <t>Pack Gift Tubes</t>
+  </si>
+  <si>
+    <t>W/House Assemble Plan with Phoebe</t>
+  </si>
+  <si>
+    <t>Continue Despatch Training Phoebe</t>
+  </si>
+  <si>
+    <t>Team training needs - identify + act</t>
+  </si>
+  <si>
+    <t>Decide on new Product lines</t>
+  </si>
+  <si>
+    <t>Confirm Building Works</t>
+  </si>
+  <si>
+    <t>Jon · Business Lead · Weekly Actions</t>
+  </si>
+  <si>
+    <t>Jon</t>
+  </si>
+  <si>
+    <t>Amazon Account Validation (VAT + Phone)</t>
+  </si>
+  <si>
+    <t>B2B - 2 key accounts/month</t>
+  </si>
+  <si>
+    <t>Contact Accountants &amp; Chase Amazon</t>
+  </si>
+  <si>
+    <t>Support Phoebe - Orders Despatch</t>
+  </si>
+  <si>
+    <t>Business Strategy &amp; Performance</t>
+  </si>
+  <si>
+    <t>Mon-Thu Practice</t>
+  </si>
+  <si>
+    <t>Teach Phoebe Invoicing</t>
+  </si>
+  <si>
+    <t>Monday Teaching</t>
+  </si>
+  <si>
+    <t>Payroll</t>
+  </si>
+  <si>
+    <t>Monday Update</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Launch New Dashboard </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monday Meeting Unveil </t>
+  </si>
+  <si>
+    <t>Finalise 2026 Product Range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GreenFingers Outstanding </t>
+  </si>
+  <si>
+    <t>Monitor International Orders</t>
+  </si>
+  <si>
+    <t>International - shipping + Amz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPS checkin </t>
+  </si>
+  <si>
+    <t>2026-W14</t>
+  </si>
+  <si>
+    <t>GlobalCheckout Setup</t>
+  </si>
+  <si>
+    <t>Bread&amp;Jam Tickets</t>
+  </si>
+  <si>
+    <t>Buy these</t>
+  </si>
+  <si>
+    <t>Checking WIth Corp Campaigns: Virgin, PIPL, SmartCurrencyExchange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email each Monday </t>
+  </si>
+  <si>
+    <t>PPC Check-in &amp; Ypdate</t>
+  </si>
+  <si>
+    <t>PPC - Blended ROAS 5x</t>
+  </si>
+  <si>
+    <t>Create Brochure (Inbox)</t>
   </si>
   <si>
     <t>Active Concerns - Rosie adds new items at Monday meeting</t>
@@ -3486,9 +3486,6 @@
     <t>Captures Recipients Thinking</t>
   </si>
   <si>
-    <t>7 posts per week</t>
-  </si>
-  <si>
     <t>3 Buyer Focused Posts</t>
   </si>
   <si>
@@ -3501,13 +3498,19 @@
     <t>Captures Brand Experience</t>
   </si>
   <si>
+    <t>Respond to Messages Comments</t>
+  </si>
+  <si>
+    <t>Within 4 Working Hours</t>
+  </si>
+  <si>
     <t>Reported in Monday Meeting</t>
   </si>
   <si>
     <t>Increased Reach + Followers</t>
   </si>
   <si>
-    <t>3 emails per week (1 promo)</t>
+    <t>Email Campaigns</t>
   </si>
   <si>
     <t>3 emails - subject line approved first</t>
@@ -4088,10 +4091,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4440,15 +4443,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FF2E5C32"/>
   </sheetPr>
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="20.140625" defaultRowHeight="39.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="39.75" customHeight="1"/>
   <cols>
-    <col min="1" max="8" width="35.7109375" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="20.140625" style="1"/>
+    <col min="1" max="8" width="44.42578125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="39.75" customHeight="1">
@@ -4463,7 +4466,7 @@
       <c r="G1" s="42"/>
       <c r="H1" s="42"/>
     </row>
-    <row r="2" spans="1:8" ht="15.95" customHeight="1">
+    <row r="2" spans="1:8" ht="11.25" customHeight="1">
       <c r="A2" s="36" t="s">
         <v>1</v>
       </c>
@@ -4501,7 +4504,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="39.75" customHeight="1">
+    <row r="4" spans="1:8" ht="36" customHeight="1">
       <c r="A4" s="6" t="s">
         <v>10</v>
       </c>
@@ -4514,7 +4517,7 @@
       <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="5" t="s">
@@ -4525,7 +4528,7 @@
       </c>
       <c r="H4" s="6"/>
     </row>
-    <row r="5" spans="1:8" ht="39.75" customHeight="1">
+    <row r="5" spans="1:8" ht="36" customHeight="1">
       <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
@@ -4538,14 +4541,14 @@
       <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>19</v>
       </c>
       <c r="H5" s="6"/>
     </row>
@@ -4560,16 +4563,16 @@
         <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>21</v>
       </c>
       <c r="H6" s="6"/>
     </row>
@@ -4577,189 +4580,119 @@
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>23</v>
-      </c>
+      <c r="G7" s="5"/>
       <c r="H7" s="6"/>
     </row>
     <row r="8" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="6"/>
+      <c r="B8" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>25</v>
-      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
       <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="6"/>
+      <c r="B9" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>27</v>
-      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
       <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="6" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
       <c r="H10" s="6"/>
     </row>
     <row r="11" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="A11" s="6"/>
+      <c r="B11" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="6" t="s">
+      <c r="A12" s="6"/>
+      <c r="B12" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>34</v>
-      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="6"/>
     </row>
     <row r="13" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="6" t="s">
+      <c r="A13" s="6"/>
+      <c r="B13" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>36</v>
-      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
       <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="6" t="s">
+      <c r="A14" s="6"/>
+      <c r="B14" s="21" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>38</v>
-      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
     </row>
@@ -4769,13 +4702,11 @@
         <v>11</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>39</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D15" s="6"/>
       <c r="E15" s="6"/>
-      <c r="F15" s="5"/>
+      <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
     </row>
@@ -4789,7 +4720,7 @@
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="5"/>
+      <c r="F16" s="6"/>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
     </row>
@@ -4803,7 +4734,7 @@
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="5"/>
+      <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
     </row>
@@ -4817,7 +4748,7 @@
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
-      <c r="F18" s="5"/>
+      <c r="F18" s="6"/>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
     </row>
@@ -4831,7 +4762,7 @@
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
-      <c r="F19" s="5"/>
+      <c r="F19" s="6"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
     </row>
@@ -4845,7 +4776,7 @@
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
-      <c r="F20" s="5"/>
+      <c r="F20" s="6"/>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
     </row>
@@ -4859,7 +4790,7 @@
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
-      <c r="F21" s="5"/>
+      <c r="F21" s="6"/>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
     </row>
@@ -4873,7 +4804,7 @@
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
     </row>
@@ -4887,7 +4818,7 @@
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="5"/>
+      <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
     </row>
@@ -4901,7 +4832,7 @@
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
-      <c r="F24" s="5"/>
+      <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
     </row>
@@ -4915,19 +4846,23 @@
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
-      <c r="F25" s="5"/>
+      <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
     </row>
     <row r="26" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A26" s="43"/>
-      <c r="B26" s="43"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="43"/>
+      <c r="A26" s="6"/>
+      <c r="B26" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4935,13 +4870,13 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="E4:E25" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="E4:E26" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"done,on-track,blocked,overdue"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F26" xr:uid="{FF448B2F-3CE4-4CE3-B936-F3344E3A794A}">
-      <formula1>"PPC - Blended ROAS 5x,B2B - 2 key accounts/month,International - shipping + Amz,Business Strategy &amp; Performance"</formula1>
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a Goal" error="Pick a Parent Goal from the dropdown list." sqref="F4:F26" xr:uid="{85CDD0B5-41DD-4AE7-9A41-DE69BB2082B4}">
+      <formula1>"Customer service - 4hr SLA,Order satisfaction + despatch,Stock planning,Website listings accurate,Admin &amp; Finance"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Category" error="Pick a category from the dropdown list." sqref="C4:C25" xr:uid="{F7BB392A-2390-45D1-9090-150880ECDA5F}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Category" error="Pick a category from the dropdown list." sqref="C4:C26" xr:uid="{7CD48F7F-F5B2-4620-99E8-86BB3D6A829E}">
       <formula1>"This Week,This Month,Other,Urgent"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4950,6 +4885,438 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF2E5C32"/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="39.75" customHeight="1"/>
+  <cols>
+    <col min="1" max="8" width="44.5703125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="26.1" customHeight="1">
+      <c r="A1" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+    </row>
+    <row r="2" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A2" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+    </row>
+    <row r="3" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="5"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="5"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A9" s="6"/>
+      <c r="B9" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A10" s="6"/>
+      <c r="B10" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A11" s="6"/>
+      <c r="B11" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A12" s="6"/>
+      <c r="B12" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A13" s="6"/>
+      <c r="B13" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A14" s="6"/>
+      <c r="B14" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A15" s="6"/>
+      <c r="B15" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A16" s="6"/>
+      <c r="B16" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A17" s="6"/>
+      <c r="B17" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A18" s="6"/>
+      <c r="B18" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A19" s="6"/>
+      <c r="B19" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A20" s="6"/>
+      <c r="B20" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A21" s="6"/>
+      <c r="B21" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A22" s="6"/>
+      <c r="B22" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A23" s="6"/>
+      <c r="B23" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A24" s="6"/>
+      <c r="B24" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A25" s="6"/>
+      <c r="B25" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="E4:E25" xr:uid="{00000000-0002-0000-0300-000000000000}">
+      <formula1>"done,on-track,blocked,overdue"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a Goal" error="Pick a Parent Goal from the dropdown list." sqref="F4:F25" xr:uid="{AC38FA6C-429F-4EB2-B31A-870705A524F0}">
+      <formula1>"Social Media Content,3 emails per week (1 promo),Meta UGC &amp; Creatives,Q4 campaign calendar by Aug 31,Team Support"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Category" error="Pick a category from the dropdown list." sqref="C4:C25" xr:uid="{2627C534-9878-4FF1-BD95-5C5BB730CFE0}">
+      <formula1>"This Week,This Month,Other,Urgent"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF2E5C32"/>
@@ -4963,7 +5330,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="22" customFormat="1" ht="26.1" customHeight="1">
       <c r="A1" s="39" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -4977,13 +5344,13 @@
       <c r="A2" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:8" ht="39.75" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -5016,19 +5383,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C4" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G4" s="18"/>
       <c r="H4" s="15"/>
@@ -5038,19 +5405,19 @@
         <v>10</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C5" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G5" s="18"/>
       <c r="H5" s="15"/>
@@ -5060,19 +5427,19 @@
         <v>10</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="15"/>
@@ -5082,19 +5449,19 @@
         <v>10</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G7" s="18"/>
       <c r="H7" s="15"/>
@@ -5104,19 +5471,19 @@
         <v>10</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G8" s="18"/>
       <c r="H8" s="15"/>
@@ -5126,19 +5493,19 @@
         <v>10</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G9" s="18"/>
       <c r="H9" s="15"/>
@@ -5148,19 +5515,19 @@
         <v>10</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G10" s="18"/>
       <c r="H10" s="15"/>
@@ -5170,13 +5537,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>9</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>14</v>
@@ -5188,7 +5555,7 @@
     <row r="12" spans="1:8" ht="39.75" customHeight="1">
       <c r="A12" s="15"/>
       <c r="B12" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C12" s="25" t="s">
         <v>12</v>
@@ -5202,7 +5569,7 @@
     <row r="13" spans="1:8" ht="39.75" customHeight="1">
       <c r="A13" s="15"/>
       <c r="B13" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C13" s="25" t="s">
         <v>12</v>
@@ -5216,7 +5583,7 @@
     <row r="14" spans="1:8" ht="39.75" customHeight="1">
       <c r="A14" s="15"/>
       <c r="B14" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C14" s="25" t="s">
         <v>12</v>
@@ -5230,7 +5597,7 @@
     <row r="15" spans="1:8" ht="39.75" customHeight="1">
       <c r="A15" s="15"/>
       <c r="B15" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>12</v>
@@ -5244,7 +5611,7 @@
     <row r="16" spans="1:8" ht="39.75" customHeight="1">
       <c r="A16" s="15"/>
       <c r="B16" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C16" s="25" t="s">
         <v>12</v>
@@ -5258,7 +5625,7 @@
     <row r="17" spans="1:8" ht="39.75" customHeight="1">
       <c r="A17" s="15"/>
       <c r="B17" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C17" s="25" t="s">
         <v>12</v>
@@ -5272,7 +5639,7 @@
     <row r="18" spans="1:8" ht="39.75" customHeight="1">
       <c r="A18" s="15"/>
       <c r="B18" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C18" s="25" t="s">
         <v>12</v>
@@ -5286,7 +5653,7 @@
     <row r="19" spans="1:8" ht="39.75" customHeight="1">
       <c r="A19" s="15"/>
       <c r="B19" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>12</v>
@@ -5300,7 +5667,7 @@
     <row r="20" spans="1:8" ht="39.75" customHeight="1">
       <c r="A20" s="15"/>
       <c r="B20" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>12</v>
@@ -5314,7 +5681,7 @@
     <row r="21" spans="1:8" ht="39.75" customHeight="1">
       <c r="A21" s="15"/>
       <c r="B21" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C21" s="25" t="s">
         <v>12</v>
@@ -5328,7 +5695,7 @@
     <row r="22" spans="1:8" ht="39.75" customHeight="1">
       <c r="A22" s="15"/>
       <c r="B22" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C22" s="25" t="s">
         <v>12</v>
@@ -5342,7 +5709,7 @@
     <row r="23" spans="1:8" ht="39.75" customHeight="1">
       <c r="A23" s="15"/>
       <c r="B23" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C23" s="25" t="s">
         <v>12</v>
@@ -5356,7 +5723,7 @@
     <row r="24" spans="1:8" ht="39.75" customHeight="1">
       <c r="A24" s="15"/>
       <c r="B24" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C24" s="25" t="s">
         <v>12</v>
@@ -5370,7 +5737,7 @@
     <row r="25" spans="1:8" ht="39.75" customHeight="1">
       <c r="A25" s="15"/>
       <c r="B25" s="27" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C25" s="25" t="s">
         <v>12</v>
@@ -5401,21 +5768,21 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF2E5C32"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="39.75" customHeight="1"/>
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr defaultColWidth="20.140625" defaultRowHeight="39.75" customHeight="1"/>
   <cols>
-    <col min="1" max="8" width="44.5703125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="8" width="35.7109375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="20.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="26.1" customHeight="1">
+    <row r="1" spans="1:8" ht="39.75" customHeight="1">
       <c r="A1" s="37" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -5425,7 +5792,7 @@
       <c r="G1" s="42"/>
       <c r="H1" s="42"/>
     </row>
-    <row r="2" spans="1:8" ht="39.75" customHeight="1">
+    <row r="2" spans="1:8" ht="15.95" customHeight="1">
       <c r="A2" s="36" t="s">
         <v>1</v>
       </c>
@@ -5468,21 +5835,23 @@
         <v>10</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C4" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G4" s="5"/>
+        <v>50</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="H4" s="6"/>
     </row>
     <row r="5" spans="1:8" ht="39.75" customHeight="1">
@@ -5490,21 +5859,23 @@
         <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C5" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="5"/>
+        <v>53</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>54</v>
+      </c>
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:8" ht="39.75" customHeight="1">
@@ -5512,306 +5883,380 @@
         <v>10</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C6" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G6" s="6"/>
+        <v>53</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:8" ht="39.75" customHeight="1">
       <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="21" t="s">
-        <v>54</v>
+      <c r="B7" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C7" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E7" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G7" s="6"/>
+      <c r="F7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="H7" s="6"/>
     </row>
     <row r="8" spans="1:8" ht="39.75" customHeight="1">
       <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="21" t="s">
-        <v>54</v>
+      <c r="B8" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C8" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E8" s="23" t="s">
+      <c r="D8" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>63</v>
+      <c r="F8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>60</v>
       </c>
       <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="21" t="s">
-        <v>54</v>
+      <c r="A9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C9" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="D9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>62</v>
+      </c>
       <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="21" t="s">
-        <v>54</v>
+      <c r="A10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="D10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="H10" s="6"/>
     </row>
     <row r="11" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="21" t="s">
-        <v>54</v>
+      <c r="A11" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="D11" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A12" s="6"/>
-      <c r="B12" s="21" t="s">
-        <v>54</v>
+      <c r="A12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C12" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="D12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>69</v>
+      </c>
       <c r="H12" s="6"/>
     </row>
     <row r="13" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A13" s="6"/>
-      <c r="B13" s="21" t="s">
-        <v>54</v>
+      <c r="A13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C13" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="D13" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A14" s="6"/>
-      <c r="B14" s="21" t="s">
-        <v>54</v>
+      <c r="A14" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="C14" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
+      <c r="D14" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>73</v>
+      </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
     </row>
     <row r="15" spans="1:8" ht="39.75" customHeight="1">
       <c r="A15" s="6"/>
       <c r="B15" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="6"/>
+        <v>9</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="F15" s="5"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:8" ht="39.75" customHeight="1">
       <c r="A16" s="6"/>
       <c r="B16" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C16" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="F16" s="5"/>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
     </row>
     <row r="17" spans="1:8" ht="39.75" customHeight="1">
       <c r="A17" s="6"/>
       <c r="B17" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C17" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
+      <c r="F17" s="5"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
     </row>
     <row r="18" spans="1:8" ht="39.75" customHeight="1">
       <c r="A18" s="6"/>
       <c r="B18" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C18" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="F18" s="5"/>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
     </row>
     <row r="19" spans="1:8" ht="39.75" customHeight="1">
       <c r="A19" s="6"/>
       <c r="B19" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C19" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
+      <c r="F19" s="5"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
     </row>
     <row r="20" spans="1:8" ht="39.75" customHeight="1">
       <c r="A20" s="6"/>
       <c r="B20" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C20" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
+      <c r="F20" s="5"/>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
     </row>
     <row r="21" spans="1:8" ht="39.75" customHeight="1">
       <c r="A21" s="6"/>
       <c r="B21" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C21" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
+      <c r="F21" s="5"/>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
     </row>
     <row r="22" spans="1:8" ht="39.75" customHeight="1">
       <c r="A22" s="6"/>
       <c r="B22" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C22" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
+      <c r="F22" s="5"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
     </row>
     <row r="23" spans="1:8" ht="39.75" customHeight="1">
       <c r="A23" s="6"/>
       <c r="B23" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
+      <c r="F23" s="5"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
     </row>
     <row r="24" spans="1:8" ht="39.75" customHeight="1">
       <c r="A24" s="6"/>
       <c r="B24" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C24" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
+      <c r="F24" s="5"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
     </row>
     <row r="25" spans="1:8" ht="39.75" customHeight="1">
       <c r="A25" s="6"/>
       <c r="B25" s="21" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C25" s="20" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
+      <c r="F25" s="5"/>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
+    </row>
+    <row r="26" spans="1:8" ht="39.75" customHeight="1">
+      <c r="A26" s="44"/>
+      <c r="B26" s="44"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="44"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5819,455 +6264,13 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="E4:E25" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="E4:E25" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"done,on-track,blocked,overdue"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a Goal" error="Pick a Parent Goal from the dropdown list." sqref="F4:F25" xr:uid="{AC38FA6C-429F-4EB2-B31A-870705A524F0}">
-      <formula1>"Social Media Content,3 emails per week (1 promo),Meta UGC &amp; Creatives,Q4 campaign calendar by Aug 31,Team Support"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F26" xr:uid="{FF448B2F-3CE4-4CE3-B936-F3344E3A794A}">
+      <formula1>"PPC - Blended ROAS 5x,B2B - 2 key accounts/month,International - shipping + Amz,Business Strategy &amp; Performance"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Category" error="Pick a category from the dropdown list." sqref="C4:C25" xr:uid="{2627C534-9878-4FF1-BD95-5C5BB730CFE0}">
-      <formula1>"This Week,This Month,Other,Urgent"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FF2E5C32"/>
-  </sheetPr>
-  <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="39.75" customHeight="1"/>
-  <cols>
-    <col min="1" max="8" width="44.42578125" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.85546875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A1" s="37" t="s">
-        <v>64</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-    </row>
-    <row r="2" spans="1:8" ht="11.25" customHeight="1">
-      <c r="A2" s="36" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-    </row>
-    <row r="3" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="36" customHeight="1">
-      <c r="A4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="H4" s="6"/>
-    </row>
-    <row r="5" spans="1:8" ht="36" customHeight="1">
-      <c r="A5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="6"/>
-    </row>
-    <row r="8" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A8" s="6"/>
-      <c r="B8" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-    </row>
-    <row r="9" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-    </row>
-    <row r="10" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-    </row>
-    <row r="11" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-    </row>
-    <row r="12" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A12" s="6"/>
-      <c r="B12" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-    </row>
-    <row r="13" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A13" s="6"/>
-      <c r="B13" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-    </row>
-    <row r="14" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A14" s="6"/>
-      <c r="B14" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A15" s="6"/>
-      <c r="B15" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-    </row>
-    <row r="16" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A16" s="6"/>
-      <c r="B16" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A17" s="6"/>
-      <c r="B17" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A18" s="6"/>
-      <c r="B18" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A19" s="6"/>
-      <c r="B19" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-    </row>
-    <row r="20" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A20" s="6"/>
-      <c r="B20" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A21" s="6"/>
-      <c r="B21" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-    </row>
-    <row r="22" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A22" s="6"/>
-      <c r="B22" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-    </row>
-    <row r="23" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A23" s="6"/>
-      <c r="B23" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-    </row>
-    <row r="24" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A24" s="6"/>
-      <c r="B24" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C24" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-    </row>
-    <row r="25" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A25" s="6"/>
-      <c r="B25" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-    </row>
-    <row r="26" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A26" s="6"/>
-      <c r="B26" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="E4:E26" xr:uid="{00000000-0002-0000-0400-000000000000}">
-      <formula1>"done,on-track,blocked,overdue"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a Goal" error="Pick a Parent Goal from the dropdown list." sqref="F4:F26" xr:uid="{85CDD0B5-41DD-4AE7-9A41-DE69BB2082B4}">
-      <formula1>"Customer service - 4hr SLA,Order satisfaction + despatch,Stock planning,Website listings accurate,Admin &amp; Finance"</formula1>
-    </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Category" error="Pick a category from the dropdown list." sqref="C4:C26" xr:uid="{7CD48F7F-F5B2-4620-99E8-86BB3D6A829E}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Category" error="Pick a category from the dropdown list." sqref="C4:C25" xr:uid="{F7BB392A-2390-45D1-9090-150880ECDA5F}">
       <formula1>"This Week,This Month,Other,Urgent"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6322,7 +6325,7 @@
         <v>81</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C3" s="26" t="s">
         <v>82</v>
@@ -6342,7 +6345,7 @@
         <v>85</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C4" s="26" t="s">
         <v>82</v>
@@ -6362,7 +6365,7 @@
         <v>87</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C5" s="26" t="s">
         <v>88</v>
@@ -6382,7 +6385,7 @@
         <v>90</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C6" s="26" t="s">
         <v>88</v>
@@ -15270,7 +15273,7 @@
   <sheetPr>
     <tabColor rgb="FF1E3A20"/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="39.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
@@ -15315,13 +15318,13 @@
     </row>
     <row r="3" spans="1:7" ht="39.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B3" s="4">
         <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>1089</v>
@@ -15336,13 +15339,13 @@
     </row>
     <row r="4" spans="1:7" ht="39.75" customHeight="1">
       <c r="A4" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B4" s="4">
         <v>1</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>1092</v>
@@ -15357,13 +15360,13 @@
     </row>
     <row r="5" spans="1:7" ht="39.75" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B5" s="4">
         <v>1</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>1094</v>
@@ -15378,13 +15381,13 @@
     </row>
     <row r="6" spans="1:7" ht="39.75" customHeight="1">
       <c r="A6" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B6" s="4">
         <v>2</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>1096</v>
@@ -15399,13 +15402,13 @@
     </row>
     <row r="7" spans="1:7" ht="39.75" customHeight="1">
       <c r="A7" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B7" s="4">
         <v>2</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>1098</v>
@@ -15420,13 +15423,13 @@
     </row>
     <row r="8" spans="1:7" ht="39.75" customHeight="1">
       <c r="A8" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B8" s="4">
         <v>2</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>1100</v>
@@ -15441,13 +15444,13 @@
     </row>
     <row r="9" spans="1:7" ht="39.75" customHeight="1">
       <c r="A9" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B9" s="4">
         <v>3</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>1102</v>
@@ -15462,13 +15465,13 @@
     </row>
     <row r="10" spans="1:7" ht="39.75" customHeight="1">
       <c r="A10" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B10" s="4">
         <v>3</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>1104</v>
@@ -15483,13 +15486,13 @@
     </row>
     <row r="11" spans="1:7" ht="39.75" customHeight="1">
       <c r="A11" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B11" s="4">
         <v>3</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>29</v>
+        <v>64</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>1106</v>
@@ -15504,13 +15507,13 @@
     </row>
     <row r="12" spans="1:7" ht="39.75" customHeight="1">
       <c r="A12" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B12" s="4">
         <v>4</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>1108</v>
@@ -15525,13 +15528,13 @@
     </row>
     <row r="13" spans="1:7" ht="39.75" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B13" s="4">
         <v>4</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>1110</v>
@@ -15546,13 +15549,13 @@
     </row>
     <row r="14" spans="1:7" ht="39.75" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="B14" s="4">
         <v>4</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>1112</v>
@@ -15576,13 +15579,13 @@
     </row>
     <row r="16" spans="1:7" ht="39.75" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B16" s="4">
         <v>1</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>1114</v>
@@ -15597,13 +15600,13 @@
     </row>
     <row r="17" spans="1:7" ht="39.75" customHeight="1">
       <c r="A17" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B17" s="4">
         <v>1</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>1116</v>
@@ -15618,13 +15621,13 @@
     </row>
     <row r="18" spans="1:7" ht="39.75" customHeight="1">
       <c r="A18" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B18" s="4">
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>1118</v>
@@ -15639,13 +15642,13 @@
     </row>
     <row r="19" spans="1:7" ht="39.75" customHeight="1">
       <c r="A19" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B19" s="4">
         <v>2</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>1120</v>
@@ -15660,13 +15663,13 @@
     </row>
     <row r="20" spans="1:7" ht="39.75" customHeight="1">
       <c r="A20" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B20" s="4">
         <v>2</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>1122</v>
@@ -15681,13 +15684,13 @@
     </row>
     <row r="21" spans="1:7" ht="39.75" customHeight="1">
       <c r="A21" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B21" s="4">
         <v>2</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>1124</v>
@@ -15702,7 +15705,7 @@
     </row>
     <row r="22" spans="1:7" ht="39.75" customHeight="1">
       <c r="A22" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B22" s="4">
         <v>3</v>
@@ -15723,7 +15726,7 @@
     </row>
     <row r="23" spans="1:7" ht="39.75" customHeight="1">
       <c r="A23" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B23" s="4">
         <v>3</v>
@@ -15744,7 +15747,7 @@
     </row>
     <row r="24" spans="1:7" ht="39.75" customHeight="1">
       <c r="A24" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B24" s="4">
         <v>3</v>
@@ -15765,7 +15768,7 @@
     </row>
     <row r="25" spans="1:7" ht="39.75" customHeight="1">
       <c r="A25" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B25" s="4">
         <v>3</v>
@@ -15786,13 +15789,13 @@
     </row>
     <row r="26" spans="1:7" ht="39.75" customHeight="1">
       <c r="A26" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B26" s="4">
         <v>4</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>1133</v>
@@ -15807,13 +15810,13 @@
     </row>
     <row r="27" spans="1:7" ht="39.75" customHeight="1">
       <c r="A27" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B27" s="4">
         <v>4</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>1134</v>
@@ -15828,13 +15831,13 @@
     </row>
     <row r="28" spans="1:7" ht="39.75" customHeight="1">
       <c r="A28" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B28" s="4">
         <v>4</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>1136</v>
@@ -15849,13 +15852,13 @@
     </row>
     <row r="29" spans="1:7" ht="39.75" customHeight="1">
       <c r="A29" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B29" s="4">
         <v>4</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>1138</v>
@@ -15870,13 +15873,13 @@
     </row>
     <row r="30" spans="1:7" ht="39.75" customHeight="1">
       <c r="A30" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B30" s="4">
         <v>4</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>1140</v>
@@ -15891,7 +15894,7 @@
     </row>
     <row r="31" spans="1:7" ht="39.75" customHeight="1">
       <c r="A31" s="11" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B31" s="50"/>
       <c r="C31" s="50"/>
@@ -15902,13 +15905,13 @@
     </row>
     <row r="32" spans="1:7" ht="39.75" customHeight="1">
       <c r="A32" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B32" s="4">
         <v>1</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>1142</v>
@@ -15923,19 +15926,19 @@
     </row>
     <row r="33" spans="1:7" ht="39.75" customHeight="1">
       <c r="A33" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B33" s="4">
         <v>1</v>
       </c>
       <c r="C33" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>1144</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="E33" s="6" t="s">
         <v>1145</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>1146</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>1091</v>
@@ -15944,19 +15947,19 @@
     </row>
     <row r="34" spans="1:7" ht="39.75" customHeight="1">
       <c r="A34" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B34" s="4">
         <v>1</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>1144</v>
+        <v>28</v>
       </c>
       <c r="D34" s="5" t="s">
+        <v>1146</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>1147</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>1148</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>1091</v>
@@ -15965,38 +15968,40 @@
     </row>
     <row r="35" spans="1:7" ht="39.75" customHeight="1">
       <c r="A35" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B35" s="4">
         <v>1</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>1144</v>
+        <v>28</v>
       </c>
       <c r="D35" s="5" t="s">
+        <v>1148</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>1149</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>1150</v>
-      </c>
-      <c r="F35" s="7"/>
+      <c r="F35" s="7" t="s">
+        <v>1091</v>
+      </c>
       <c r="G35" s="6"/>
     </row>
     <row r="36" spans="1:7" ht="39.75" customHeight="1">
       <c r="A36" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B36" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>1150</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>1151</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>1152</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>1153</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>1091</v>
@@ -16005,19 +16010,19 @@
     </row>
     <row r="37" spans="1:7" ht="39.75" customHeight="1">
       <c r="A37" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B37" s="4">
         <v>2</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="D37" s="5" t="s">
+        <v>1153</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>1154</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>1155</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>1091</v>
@@ -16026,16 +16031,16 @@
     </row>
     <row r="38" spans="1:7" ht="39.75" customHeight="1">
       <c r="A38" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B38" s="4">
         <v>2</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>1149</v>
+        <v>1155</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>1156</v>
@@ -16047,19 +16052,19 @@
     </row>
     <row r="39" spans="1:7" ht="39.75" customHeight="1">
       <c r="A39" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B39" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C39" s="5" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>1150</v>
+      </c>
+      <c r="E39" s="6" t="s">
         <v>1157</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>1158</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>1159</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>1091</v>
@@ -16068,19 +16073,19 @@
     </row>
     <row r="40" spans="1:7" ht="39.75" customHeight="1">
       <c r="A40" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B40" s="4">
         <v>3</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D40" s="5" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>1160</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>1161</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>1091</v>
@@ -16089,65 +16094,63 @@
     </row>
     <row r="41" spans="1:7" ht="39.75" customHeight="1">
       <c r="A41" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B41" s="4">
         <v>3</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D41" s="5" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>1162</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>1163</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>1091</v>
       </c>
-      <c r="G41" s="6" t="s">
-        <v>1164</v>
-      </c>
+      <c r="G41" s="6"/>
     </row>
     <row r="42" spans="1:7" ht="39.75" customHeight="1">
       <c r="A42" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B42" s="4">
         <v>3</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>1091</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="39.75" customHeight="1">
       <c r="A43" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B43" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C43" s="5" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>1166</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>1167</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>1168</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>1169</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>1091</v>
@@ -16156,19 +16159,19 @@
     </row>
     <row r="44" spans="1:7" ht="39.75" customHeight="1">
       <c r="A44" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B44" s="4">
         <v>4</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="D44" s="5" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>1170</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>1171</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>1091</v>
@@ -16177,19 +16180,19 @@
     </row>
     <row r="45" spans="1:7" ht="39.75" customHeight="1">
       <c r="A45" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B45" s="4">
         <v>4</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>1091</v>
@@ -16198,19 +16201,19 @@
     </row>
     <row r="46" spans="1:7" ht="39.75" customHeight="1">
       <c r="A46" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B46" s="4">
         <v>4</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="D46" s="5" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>1172</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>1173</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>1091</v>
@@ -16219,19 +16222,19 @@
     </row>
     <row r="47" spans="1:7" ht="39.75" customHeight="1">
       <c r="A47" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B47" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>61</v>
+        <v>1168</v>
       </c>
       <c r="D47" s="5" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>1174</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>1175</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>1091</v>
@@ -16240,19 +16243,19 @@
     </row>
     <row r="48" spans="1:7" ht="39.75" customHeight="1">
       <c r="A48" s="12" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="B48" s="4">
         <v>5</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="D48" s="5" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>1176</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>1175</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>1091</v>
@@ -16260,52 +16263,52 @@
       <c r="G48" s="6"/>
     </row>
     <row r="49" spans="1:7" ht="39.75" customHeight="1">
-      <c r="A49" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="B49" s="50"/>
-      <c r="C49" s="50"/>
-      <c r="D49" s="50"/>
-      <c r="E49" s="50"/>
-      <c r="F49" s="50"/>
-      <c r="G49" s="50"/>
+      <c r="A49" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B49" s="4">
+        <v>5</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>1176</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>1091</v>
+      </c>
+      <c r="G49" s="6"/>
     </row>
     <row r="50" spans="1:7" ht="39.75" customHeight="1">
-      <c r="A50" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B50" s="4">
-        <v>1</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>1177</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>1178</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>1091</v>
-      </c>
-      <c r="G50" s="6"/>
+      <c r="A50" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B50" s="50"/>
+      <c r="C50" s="50"/>
+      <c r="D50" s="50"/>
+      <c r="E50" s="50"/>
+      <c r="F50" s="50"/>
+      <c r="G50" s="50"/>
     </row>
     <row r="51" spans="1:7" ht="39.75" customHeight="1">
       <c r="A51" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B51" s="4">
         <v>1</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="D51" s="5" t="s">
+        <v>1179</v>
+      </c>
+      <c r="E51" s="6" t="s">
         <v>1180</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>1181</v>
       </c>
       <c r="F51" s="7" t="s">
         <v>1091</v>
@@ -16314,19 +16317,19 @@
     </row>
     <row r="52" spans="1:7" ht="39.75" customHeight="1">
       <c r="A52" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B52" s="4">
         <v>1</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="D52" s="5" t="s">
+        <v>1181</v>
+      </c>
+      <c r="E52" s="6" t="s">
         <v>1182</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>1183</v>
       </c>
       <c r="F52" s="7" t="s">
         <v>1091</v>
@@ -16335,19 +16338,19 @@
     </row>
     <row r="53" spans="1:7" ht="39.75" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B53" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>67</v>
+        <v>1178</v>
       </c>
       <c r="D53" s="5" t="s">
+        <v>1183</v>
+      </c>
+      <c r="E53" s="6" t="s">
         <v>1184</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>1185</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>1091</v>
@@ -16356,19 +16359,19 @@
     </row>
     <row r="54" spans="1:7" ht="39.75" customHeight="1">
       <c r="A54" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B54" s="4">
         <v>2</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="D54" s="5" t="s">
+        <v>1185</v>
+      </c>
+      <c r="E54" s="6" t="s">
         <v>1186</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>1187</v>
       </c>
       <c r="F54" s="7" t="s">
         <v>1091</v>
@@ -16377,19 +16380,19 @@
     </row>
     <row r="55" spans="1:7" ht="39.75" customHeight="1">
       <c r="A55" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B55" s="4">
         <v>2</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="D55" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="E55" s="6" t="s">
         <v>1188</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>1189</v>
       </c>
       <c r="F55" s="7" t="s">
         <v>1091</v>
@@ -16398,19 +16401,19 @@
     </row>
     <row r="56" spans="1:7" ht="39.75" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B56" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="D56" s="5" t="s">
+        <v>1189</v>
+      </c>
+      <c r="E56" s="6" t="s">
         <v>1190</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>1191</v>
       </c>
       <c r="F56" s="7" t="s">
         <v>1091</v>
@@ -16419,19 +16422,19 @@
     </row>
     <row r="57" spans="1:7" ht="39.75" customHeight="1">
       <c r="A57" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B57" s="4">
         <v>3</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D57" s="5" t="s">
+        <v>1191</v>
+      </c>
+      <c r="E57" s="6" t="s">
         <v>1192</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>1193</v>
       </c>
       <c r="F57" s="7" t="s">
         <v>1091</v>
@@ -16440,19 +16443,19 @@
     </row>
     <row r="58" spans="1:7" ht="39.75" customHeight="1">
       <c r="A58" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B58" s="4">
         <v>3</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D58" s="5" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E58" s="6" t="s">
         <v>1194</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>1195</v>
       </c>
       <c r="F58" s="7" t="s">
         <v>1091</v>
@@ -16461,19 +16464,19 @@
     </row>
     <row r="59" spans="1:7" ht="39.75" customHeight="1">
       <c r="A59" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B59" s="4">
         <v>3</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D59" s="5" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E59" s="6" t="s">
         <v>1196</v>
-      </c>
-      <c r="E59" s="6" t="s">
-        <v>1197</v>
       </c>
       <c r="F59" s="7" t="s">
         <v>1091</v>
@@ -16482,19 +16485,19 @@
     </row>
     <row r="60" spans="1:7" ht="39.75" customHeight="1">
       <c r="A60" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B60" s="4">
         <v>3</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D60" s="5" t="s">
+        <v>1197</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>1198</v>
-      </c>
-      <c r="E60" s="6" t="s">
-        <v>1197</v>
       </c>
       <c r="F60" s="7" t="s">
         <v>1091</v>
@@ -16503,19 +16506,19 @@
     </row>
     <row r="61" spans="1:7" ht="39.75" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B61" s="4">
         <v>3</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>1199</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>1091</v>
@@ -16524,19 +16527,19 @@
     </row>
     <row r="62" spans="1:7" ht="39.75" customHeight="1">
       <c r="A62" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B62" s="4">
         <v>3</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="D62" s="5" t="s">
+        <v>1200</v>
+      </c>
+      <c r="E62" s="6" t="s">
         <v>1201</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>1195</v>
       </c>
       <c r="F62" s="7" t="s">
         <v>1091</v>
@@ -16545,19 +16548,19 @@
     </row>
     <row r="63" spans="1:7" ht="39.75" customHeight="1">
       <c r="A63" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B63" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C63" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D63" s="5" t="s">
         <v>1202</v>
       </c>
-      <c r="D63" s="5" t="s">
-        <v>1203</v>
-      </c>
       <c r="E63" s="6" t="s">
-        <v>1204</v>
+        <v>1196</v>
       </c>
       <c r="F63" s="7" t="s">
         <v>1091</v>
@@ -16566,19 +16569,19 @@
     </row>
     <row r="64" spans="1:7" ht="39.75" customHeight="1">
       <c r="A64" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B64" s="4">
         <v>4</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="D64" s="5" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E64" s="6" t="s">
         <v>1205</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>1206</v>
       </c>
       <c r="F64" s="7" t="s">
         <v>1091</v>
@@ -16587,19 +16590,19 @@
     </row>
     <row r="65" spans="1:7" ht="39.75" customHeight="1">
       <c r="A65" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B65" s="4">
         <v>4</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="D65" s="5" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E65" s="6" t="s">
         <v>1207</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>1208</v>
       </c>
       <c r="F65" s="7" t="s">
         <v>1091</v>
@@ -16608,19 +16611,19 @@
     </row>
     <row r="66" spans="1:7" ht="39.75" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B66" s="4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>72</v>
+        <v>1203</v>
       </c>
       <c r="D66" s="5" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E66" s="6" t="s">
         <v>1209</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>1210</v>
       </c>
       <c r="F66" s="7" t="s">
         <v>1091</v>
@@ -16629,66 +16632,87 @@
     </row>
     <row r="67" spans="1:7" ht="39.75" customHeight="1">
       <c r="A67" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B67" s="4">
         <v>5</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="D67" s="5" t="s">
+        <v>1210</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>1211</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>1212</v>
       </c>
       <c r="F67" s="7" t="s">
         <v>1091</v>
       </c>
-      <c r="G67" s="43"/>
+      <c r="G67" s="6"/>
     </row>
     <row r="68" spans="1:7" ht="39.75" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B68" s="4">
         <v>5</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="D68" s="5" t="s">
+        <v>1212</v>
+      </c>
+      <c r="E68" s="6" t="s">
         <v>1213</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>1214</v>
       </c>
       <c r="F68" s="7" t="s">
         <v>1091</v>
       </c>
-      <c r="G68" s="43"/>
+      <c r="G68" s="44"/>
     </row>
     <row r="69" spans="1:7" ht="39.75" customHeight="1">
       <c r="A69" s="14" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="B69" s="4">
         <v>5</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="D69" s="5" t="s">
+        <v>1214</v>
+      </c>
+      <c r="E69" s="6" t="s">
         <v>1215</v>
-      </c>
-      <c r="E69" s="6" t="s">
-        <v>1216</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>1091</v>
       </c>
-      <c r="G69" s="43"/>
+      <c r="G69" s="44"/>
+    </row>
+    <row r="70" spans="1:7" ht="39.75" customHeight="1">
+      <c r="A70" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B70" s="4">
+        <v>5</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>1216</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>1217</v>
+      </c>
+      <c r="F70" s="7" t="s">
+        <v>1091</v>
+      </c>
+      <c r="G70" s="44"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="Jy0Ou4hMhargRxS3iD5poxO83LkBmZ6obIKLHr0IBM/LxSDXktKFAvVqbfEvCX4A6zFnznmuyVN0wZuo+tgcEQ==" saltValue="BrJE6x/3GqnJcH6AnFSCWA==" spinCount="100000" sheet="1"/>
@@ -16696,7 +16720,7 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="F3:F69" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="F3:F70" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"active,done,paused"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix all data pipeline issues + add Flight Check + /data-confidence command
Build script fixes:
- build-adspend-cache.py: fix Google Ads column names (Performance: Clicks,
  Conversions: Conversions, Cost: Amount spend) — clicks were reading as 0
- build-marketing-cache.py: graceful exit on missing TYPEFORM_TOKEN (was crashing)
- build-bom-cache.py: add ONEDRIVE_BOM_URL support for GitHub Actions
- GitHub Actions: add continue-on-error to all data steps so a single failure
  never blocks the commit; BoM step now uses ONEDRIVE_BOM_URL secret

New skill: dashboard-data-confidence.skill
- Invoke as /dashboard-data-confidence in any Claude session
- Reads all cache timestamps, checks GitHub Actions last run
- Produces confidence rating per source with age and action items

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Final Data Files/Team Pulse/EDEN_CO_Weekly_Status.xlsx
+++ b/Final Data Files/Team Pulse/EDEN_CO_Weekly_Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bf0016d8e2d976c3/eden-co-brain/data/ceo dashboard/build/Final Data Files/Team Pulse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="601" documentId="11_5BE35CD9EAE0455C5359B5B6448765289977FBF5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85EE60EC-E571-4658-A8FB-0C4FAE23B813}"/>
+  <xr:revisionPtr revIDLastSave="602" documentId="11_5BE35CD9EAE0455C5359B5B6448765289977FBF5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FDC646E-ED6F-4C3E-BA77-CDD5219932D1}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="18980" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Phoebe" sheetId="5" r:id="rId1"/>
@@ -4138,6 +4138,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4153,9 +4156,6 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4522,7 +4522,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="45"/>
@@ -4534,7 +4534,7 @@
       <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="11.25" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="45"/>
@@ -4964,7 +4964,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26.1" customHeight="1">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="40" t="s">
         <v>23</v>
       </c>
       <c r="B1" s="45"/>
@@ -4976,7 +4976,7 @@
       <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="45"/>
@@ -5396,19 +5396,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="22" customFormat="1" ht="26.1" customHeight="1">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="41" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="46"/>
@@ -5848,7 +5848,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="40" t="s">
         <v>47</v>
       </c>
       <c r="B1" s="45"/>
@@ -5860,7 +5860,7 @@
       <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="15.95" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="45"/>
@@ -6358,7 +6358,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="44" t="s">
         <v>74</v>
       </c>
       <c r="B1" s="48"/>
@@ -15394,7 +15394,7 @@
       <c r="C2" s="18">
         <v>127</v>
       </c>
-      <c r="D2" s="44">
+      <c r="D2" s="38">
         <v>46111</v>
       </c>
       <c r="E2" s="19">
@@ -15411,7 +15411,7 @@
       <c r="C3" s="19">
         <v>313</v>
       </c>
-      <c r="D3" s="44">
+      <c r="D3" s="38">
         <v>46111</v>
       </c>
       <c r="E3" s="19">
@@ -15428,7 +15428,7 @@
       <c r="C4" s="19">
         <v>0</v>
       </c>
-      <c r="D4" s="44">
+      <c r="D4" s="38">
         <v>46112</v>
       </c>
       <c r="E4" s="19">
@@ -15445,7 +15445,7 @@
       <c r="C5" s="19">
         <v>0</v>
       </c>
-      <c r="D5" s="44">
+      <c r="D5" s="38">
         <v>46111</v>
       </c>
       <c r="E5" s="19">
@@ -15462,7 +15462,7 @@
       <c r="C6" s="19">
         <v>0</v>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="38">
         <v>46111</v>
       </c>
       <c r="E6" s="19">
@@ -15479,7 +15479,7 @@
       <c r="C7" s="19">
         <v>555</v>
       </c>
-      <c r="D7" s="44">
+      <c r="D7" s="38">
         <v>46111</v>
       </c>
       <c r="E7" s="19">
@@ -15496,7 +15496,7 @@
       <c r="C8" s="19">
         <v>40</v>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="38">
         <v>46111</v>
       </c>
       <c r="E8" s="19">
@@ -15513,7 +15513,7 @@
       <c r="C9" s="19">
         <v>200</v>
       </c>
-      <c r="D9" s="44">
+      <c r="D9" s="38">
         <v>46111</v>
       </c>
       <c r="E9" s="19">
@@ -15549,7 +15549,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26.1" customHeight="1">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="40" t="s">
         <v>1101</v>
       </c>
       <c r="B1" s="45"/>

</xml_diff>